<commit_message>
Add a features slot and put the work back in the announcement opener
Briefs carry a features list (signed, numbered, free worldwide shipping,
plus bespoke items). Emails render it as a FEATURES block; posts as one
line of short sentences. The announcement opener names the work again.
The hook is about the work only; templates place the beneficiary, medium
and features. Spreadsheet updated to match.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KCpXfXvgVaMZkSdhMYLgwy
</commit_message>
<xml_diff>
--- a/tool/instagram-set.xlsx
+++ b/tool/instagram-set.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -787,196 +787,281 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>feature_1</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Signed by the artist</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>the standard three; clear a cell to drop it</t>
+        </is>
+      </c>
+    </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>feature_2</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Individually numbered</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>feature_3</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Free worldwide shipping</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>feature_4</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr"/>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>bespoke, e.g. Hand-finished by the artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>feature_5</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr"/>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>bespoke, e.g. Available individually or as a set</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>Fragments, written once per release</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="128" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="27" ht="128" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>bio</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>Grayson Perry has long been one of the most distinctive voices in contemporary British art.
 Working across ceramics, tapestry, print and sculpture, his practice examines identity, class, and gender in modern society. Drawing on autobiography as well as social observation, Grayson often pairs the decorative language of traditional craft with direct commentary on the structures and contradictions that shape everyday life.</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr">
         <is>
           <t>2 to 3 sentences on the artist, third person, no handle. Coming Soon only.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="48" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="28" ht="48" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>hook</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>Created exclusively for the Foundling Museum, this edition portrays a child as a symbol of modern youth, exploring how technology shapes today's generations and supporting the museum's mission to celebrate children in care.</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>1 to 2 sentences on the work; the same hook the email uses. Announcement only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="48" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>The Changeling portrays a child as a symbol of modern youth, exploring how technology shapes today's generations. Grayson describes the work as intentionally 'quite disturbing', a changeling reimagined for the digital age.</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>1 to 2 sentences about the work only; the same hook the email uses. The templates place the beneficiary, the medium and the features.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="48" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>making</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>To create the edition, our printmakers at Make-Ready (@make__ready) translated a new design into a 9-colour silkscreen, capturing the vivid detail of Grayson's drawing style.</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="C29" s="8" t="inlineStr">
         <is>
           <t>one sentence on how it was made, naming Make-Ready. Sustain only.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="32" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
+    <row r="30" ht="32" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>quote</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B30" s="7" t="inlineStr">
         <is>
           <t>Beauty and seriousness are perhaps the most shocking tactics left to artists these days.</t>
         </is>
       </c>
-      <c r="C25" s="8" t="inlineStr">
+      <c r="C30" s="8" t="inlineStr">
         <is>
           <t>verbatim, a complete sentence, or blank to skip the second sustain post</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="6" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>Derived (formulas, do not edit)</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>named</t>
         </is>
       </c>
-      <c r="B28" s="9">
+      <c r="B33" s="9">
         <f>$B$4&amp;IF($B$5="","", " (@"&amp;$B$5&amp;")")</f>
         <v/>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>artist with handle</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>work</t>
-        </is>
-      </c>
-      <c r="B29" s="9">
-        <f>IF($B$9="yes","the "&amp;$B$8&amp;" series","‘"&amp;$B$8&amp;"’")</f>
-        <v/>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>the title in quotes, or the series</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>Work</t>
-        </is>
-      </c>
-      <c r="B30" s="9">
-        <f>UPPER(LEFT($B$29,1))&amp;MID($B$29,2,999)</f>
-        <v/>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>the same, capitalised for the start of a sentence</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>beneficiary_tagged</t>
-        </is>
-      </c>
-      <c r="B31" s="9">
-        <f>IF($B$18="","",$B$18&amp;IF($B$19="",""," (@"&amp;$B$19&amp;")"))</f>
-        <v/>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>beneficiary with handle</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="80" customHeight="1">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>bio_tagged</t>
-        </is>
-      </c>
-      <c r="B32" s="9">
-        <f>IF($B$5="",$B$22,SUBSTITUTE($B$22,$B$4,$B$28,1))</f>
-        <v/>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>the bio with the handle after the first mention of the name</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="48" customHeight="1">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>hook_tagged</t>
-        </is>
-      </c>
-      <c r="B33" s="9">
-        <f>IF($B$31="",$B$23,SUBSTITUTE($B$23,$B$18,$B$31,1))</f>
-        <v/>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>the hook with the beneficiary tagged</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
+          <t>work</t>
+        </is>
+      </c>
+      <c r="B34" s="9">
+        <f>IF($B$9="yes","the "&amp;$B$8&amp;" series","‘"&amp;$B$8&amp;"’")</f>
+        <v/>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>the title in quotes, or the series</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="B35" s="9">
+        <f>UPPER(LEFT($B$34,1))&amp;MID($B$34,2,999)</f>
+        <v/>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>the same, capitalised for the start of a sentence</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>beneficiary_tagged</t>
+        </is>
+      </c>
+      <c r="B36" s="9">
+        <f>IF($B$18="","",$B$18&amp;IF($B$19="",""," (@"&amp;$B$19&amp;")"))</f>
+        <v/>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>beneficiary with handle</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="80" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>bio_tagged</t>
+        </is>
+      </c>
+      <c r="B37" s="9">
+        <f>IF($B$5="",$B$27,SUBSTITUTE($B$27,$B$4,$B$33,1))</f>
+        <v/>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>the bio with the handle after the first mention of the name</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="48" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>hook_tagged</t>
+        </is>
+      </c>
+      <c r="B38" s="9">
+        <f>IF($B$36="",$B$28,SUBSTITUTE($B$28,$B$18,$B$36,1))</f>
+        <v/>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>the hook with the beneficiary tagged, if it names one</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>features</t>
+        </is>
+      </c>
+      <c r="B39" s="9">
+        <f>$B$20&amp;IF($B$21="","",". "&amp;$B$21)&amp;IF($B$22="","",". "&amp;$B$22)&amp;IF($B$23="","",". "&amp;$B$23)&amp;IF($B$24="","",". "&amp;$B$24)&amp;"."</f>
+        <v/>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>the features as one line, for the posts</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
           <t>hook_names_beneficiary</t>
         </is>
       </c>
-      <c r="B34" s="9">
-        <f>IF($B$18="",FALSE,ISNUMBER(SEARCH($B$18,$B$23)))</f>
-        <v/>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="B40" s="9">
+        <f>IF($B$18="",FALSE,ISNUMBER(SEARCH($B$18,$B$28)))</f>
+        <v/>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>TRUE when the hook already names the beneficiary, so the edition line will not</t>
         </is>
@@ -993,7 +1078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1044,7 +1129,7 @@
         </is>
       </c>
       <c r="C4" s="9">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B4,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$28),"{work}",Inputs!$B$29),"{Work}",Inputs!$B$30),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$31),"{quote}",Inputs!$B$25),"{hashtag}",Inputs!$B$6)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B4,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$33),"{work}",Inputs!$B$34),"{Work}",Inputs!$B$35),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$36),"{quote}",Inputs!$B$30),"{hashtag}",Inputs!$B$6),"{features}",Inputs!$B$39)</f>
         <v/>
       </c>
     </row>
@@ -1060,7 +1145,7 @@
         </is>
       </c>
       <c r="C5" s="9">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$28),"{work}",Inputs!$B$29),"{Work}",Inputs!$B$30),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$31),"{quote}",Inputs!$B$25),"{hashtag}",Inputs!$B$6)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B5,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$33),"{work}",Inputs!$B$34),"{Work}",Inputs!$B$35),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$36),"{quote}",Inputs!$B$30),"{hashtag}",Inputs!$B$6),"{features}",Inputs!$B$39)</f>
         <v/>
       </c>
     </row>
@@ -1076,7 +1161,7 @@
         </is>
       </c>
       <c r="C6" s="9">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$28),"{work}",Inputs!$B$29),"{Work}",Inputs!$B$30),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$31),"{quote}",Inputs!$B$25),"{hashtag}",Inputs!$B$6)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$33),"{work}",Inputs!$B$34),"{Work}",Inputs!$B$35),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$36),"{quote}",Inputs!$B$30),"{hashtag}",Inputs!$B$6),"{features}",Inputs!$B$39)</f>
         <v/>
       </c>
     </row>
@@ -1092,7 +1177,7 @@
         </is>
       </c>
       <c r="C7" s="9">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$28),"{work}",Inputs!$B$29),"{Work}",Inputs!$B$30),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$31),"{quote}",Inputs!$B$25),"{hashtag}",Inputs!$B$6)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$33),"{work}",Inputs!$B$34),"{Work}",Inputs!$B$35),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$36),"{quote}",Inputs!$B$30),"{hashtag}",Inputs!$B$6),"{features}",Inputs!$B$39)</f>
         <v/>
       </c>
     </row>
@@ -1108,7 +1193,7 @@
         </is>
       </c>
       <c r="C8" s="9">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B8,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$28),"{work}",Inputs!$B$29),"{Work}",Inputs!$B$30),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$31),"{quote}",Inputs!$B$25),"{hashtag}",Inputs!$B$6)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B8,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$33),"{work}",Inputs!$B$34),"{Work}",Inputs!$B$35),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$36),"{quote}",Inputs!$B$30),"{hashtag}",Inputs!$B$6),"{features}",Inputs!$B$39)</f>
         <v/>
       </c>
     </row>
@@ -1124,7 +1209,7 @@
         </is>
       </c>
       <c r="C9" s="9">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B9,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$28),"{work}",Inputs!$B$29),"{Work}",Inputs!$B$30),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$31),"{quote}",Inputs!$B$25),"{hashtag}",Inputs!$B$6)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B9,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$33),"{work}",Inputs!$B$34),"{Work}",Inputs!$B$35),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$36),"{quote}",Inputs!$B$30),"{hashtag}",Inputs!$B$6),"{features}",Inputs!$B$39)</f>
         <v/>
       </c>
     </row>
@@ -1140,7 +1225,7 @@
         </is>
       </c>
       <c r="C10" s="9">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B10,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$28),"{work}",Inputs!$B$29),"{Work}",Inputs!$B$30),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$31),"{quote}",Inputs!$B$25),"{hashtag}",Inputs!$B$6)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B10,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$33),"{work}",Inputs!$B$34),"{Work}",Inputs!$B$35),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$36),"{quote}",Inputs!$B$30),"{hashtag}",Inputs!$B$6),"{features}",Inputs!$B$39)</f>
         <v/>
       </c>
     </row>
@@ -1156,7 +1241,7 @@
         </is>
       </c>
       <c r="C11" s="9">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B11,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$28),"{work}",Inputs!$B$29),"{Work}",Inputs!$B$30),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$31),"{quote}",Inputs!$B$25),"{hashtag}",Inputs!$B$6)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B11,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$33),"{work}",Inputs!$B$34),"{Work}",Inputs!$B$35),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$36),"{quote}",Inputs!$B$30),"{hashtag}",Inputs!$B$6),"{features}",Inputs!$B$39)</f>
         <v/>
       </c>
     </row>
@@ -1172,7 +1257,7 @@
         </is>
       </c>
       <c r="C12" s="9">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B12,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$28),"{work}",Inputs!$B$29),"{Work}",Inputs!$B$30),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$31),"{quote}",Inputs!$B$25),"{hashtag}",Inputs!$B$6)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B12,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$33),"{work}",Inputs!$B$34),"{Work}",Inputs!$B$35),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$36),"{quote}",Inputs!$B$30),"{hashtag}",Inputs!$B$6),"{features}",Inputs!$B$39)</f>
         <v/>
       </c>
     </row>
@@ -1188,167 +1273,151 @@
         </is>
       </c>
       <c r="C13" s="9">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B13,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$28),"{work}",Inputs!$B$29),"{Work}",Inputs!$B$30),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$31),"{quote}",Inputs!$B$25),"{hashtag}",Inputs!$B$6)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B13,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$33),"{work}",Inputs!$B$34),"{Work}",Inputs!$B$35),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$36),"{quote}",Inputs!$B$30),"{hashtag}",Inputs!$B$6),"{features}",Inputs!$B$39)</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>edition line</t>
+          <t>features line</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Signed by the artist and individually numbered.</t>
+          <t>{features}</t>
         </is>
       </c>
       <c r="C14" s="9">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B14,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$28),"{work}",Inputs!$B$29),"{Work}",Inputs!$B$30),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$31),"{quote}",Inputs!$B$25),"{hashtag}",Inputs!$B$6)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B14,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$33),"{work}",Inputs!$B$34),"{Work}",Inputs!$B$35),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$36),"{quote}",Inputs!$B$30),"{hashtag}",Inputs!$B$6),"{features}",Inputs!$B$39)</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>edition line, several works</t>
+          <t>beneficiary line</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Each print is signed by the artist and individually numbered.</t>
+          <t>Released in support of {beneficiary_tagged}.</t>
         </is>
       </c>
       <c r="C15" s="9">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B15,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$28),"{work}",Inputs!$B$29),"{Work}",Inputs!$B$30),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$31),"{quote}",Inputs!$B$25),"{hashtag}",Inputs!$B$6)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B15,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$33),"{work}",Inputs!$B$34),"{Work}",Inputs!$B$35),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$36),"{quote}",Inputs!$B$30),"{hashtag}",Inputs!$B$6),"{features}",Inputs!$B$39)</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>beneficiary line</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Released in support of {beneficiary_tagged}.</t>
+          <t>Closes {close_date} at {close_time}.</t>
         </is>
       </c>
       <c r="C16" s="9">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B16,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$28),"{work}",Inputs!$B$29),"{Work}",Inputs!$B$30),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$31),"{quote}",Inputs!$B$25),"{hashtag}",Inputs!$B$6)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B16,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$33),"{work}",Inputs!$B$34),"{Work}",Inputs!$B$35),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$36),"{quote}",Inputs!$B$30),"{hashtag}",Inputs!$B$6),"{features}",Inputs!$B$39)</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>action before launch, timed</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Closes {close_date} at {close_time}.</t>
+          <t>Available for {window} from {launch_time} on {launch_date}. Link in bio to get updates.</t>
         </is>
       </c>
       <c r="C17" s="9">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B17,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$28),"{work}",Inputs!$B$29),"{Work}",Inputs!$B$30),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$31),"{quote}",Inputs!$B$25),"{hashtag}",Inputs!$B$6)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B17,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$33),"{work}",Inputs!$B$34),"{Work}",Inputs!$B$35),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$36),"{quote}",Inputs!$B$30),"{hashtag}",Inputs!$B$6),"{features}",Inputs!$B$39)</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>action before launch, timed</t>
+          <t>action before launch, draw</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Available for {window} from {launch_time} on {launch_date}. Link in bio to get updates.</t>
+          <t>Enter the draw via our link in bio. Closes {close_date} at {close_time}.</t>
         </is>
       </c>
       <c r="C18" s="9">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B18,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$28),"{work}",Inputs!$B$29),"{Work}",Inputs!$B$30),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$31),"{quote}",Inputs!$B$25),"{hashtag}",Inputs!$B$6)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B18,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$33),"{work}",Inputs!$B$34),"{Work}",Inputs!$B$35),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$36),"{quote}",Inputs!$B$30),"{hashtag}",Inputs!$B$6),"{features}",Inputs!$B$39)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>action before launch, draw</t>
+          <t>action while open, timed</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Enter the draw via our link in bio. Closes {close_date} at {close_time}.</t>
+          <t>Link in bio to buy a print. Closes {close_date} at {close_time}.</t>
         </is>
       </c>
       <c r="C19" s="9">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B19,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$28),"{work}",Inputs!$B$29),"{Work}",Inputs!$B$30),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$31),"{quote}",Inputs!$B$25),"{hashtag}",Inputs!$B$6)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B19,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$33),"{work}",Inputs!$B$34),"{Work}",Inputs!$B$35),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$36),"{quote}",Inputs!$B$30),"{hashtag}",Inputs!$B$6),"{features}",Inputs!$B$39)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>action while open, timed</t>
+          <t>action while open, draw</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Link in bio to buy a print. Closes {close_date} at {close_time}.</t>
+          <t>Enter the draw via our link in bio. Closes {close_date} at {close_time}.</t>
         </is>
       </c>
       <c r="C20" s="9">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B20,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$28),"{work}",Inputs!$B$29),"{Work}",Inputs!$B$30),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$31),"{quote}",Inputs!$B$25),"{hashtag}",Inputs!$B$6)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B20,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$33),"{work}",Inputs!$B$34),"{Work}",Inputs!$B$35),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$36),"{quote}",Inputs!$B$30),"{hashtag}",Inputs!$B$6),"{features}",Inputs!$B$39)</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>action while open, draw</t>
+          <t>coming soon · action</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Enter the draw via our link in bio. Closes {close_date} at {close_time}.</t>
+          <t>Link in bio to get updates.</t>
         </is>
       </c>
       <c r="C21" s="9">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B21,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$28),"{work}",Inputs!$B$29),"{Work}",Inputs!$B$30),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$31),"{quote}",Inputs!$B$25),"{hashtag}",Inputs!$B$6)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B21,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$33),"{work}",Inputs!$B$34),"{Work}",Inputs!$B$35),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$36),"{quote}",Inputs!$B$30),"{hashtag}",Inputs!$B$6),"{features}",Inputs!$B$39)</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>coming soon · action</t>
+          <t>hashtag</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Link in bio to get updates.</t>
+          <t>#{hashtag}</t>
         </is>
       </c>
       <c r="C22" s="9">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B22,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$28),"{work}",Inputs!$B$29),"{Work}",Inputs!$B$30),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$31),"{quote}",Inputs!$B$25),"{hashtag}",Inputs!$B$6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>hashtag</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>#{hashtag}</t>
-        </is>
-      </c>
-      <c r="C23" s="9">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B23,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$28),"{work}",Inputs!$B$29),"{Work}",Inputs!$B$30),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$31),"{quote}",Inputs!$B$25),"{hashtag}",Inputs!$B$6)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B22,"{artist}",Inputs!$B$4),"{named}",Inputs!$B$33),"{work}",Inputs!$B$34),"{Work}",Inputs!$B$35),"{edition_phrase}",Inputs!$B$10),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$14),"{launch_time}",Inputs!$B$15),"{close_date}",Inputs!$B$16),"{close_time}",Inputs!$B$17),"{beneficiary_tagged}",Inputs!$B$36),"{quote}",Inputs!$B$30),"{hashtag}",Inputs!$B$6),"{features}",Inputs!$B$39)</f>
         <v/>
       </c>
     </row>
@@ -1463,7 +1532,7 @@
         <v/>
       </c>
       <c r="E4" s="10">
-        <f>Inputs!$B$32</f>
+        <f>Inputs!$B$37</f>
         <v/>
       </c>
       <c r="F4" s="10">
@@ -1471,7 +1540,7 @@
         <v/>
       </c>
       <c r="G4" s="10">
-        <f>Lines!$C$22</f>
+        <f>Lines!$C$21</f>
         <v/>
       </c>
       <c r="H4" s="10">
@@ -1498,7 +1567,7 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>status · hook · edition · action · hashtag</t>
+          <t>status · hook · features · action · hashtag</t>
         </is>
       </c>
       <c r="D5" s="10">
@@ -1506,19 +1575,19 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>Inputs!$B$33</f>
+        <f>Inputs!$B$38</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>IF(Inputs!$B$11&gt;1,Lines!$C$15,Lines!$C$14)&amp;IF(Inputs!$B$34,"",IF(Inputs!$B$31="",""," "&amp;Lines!$C$16))</f>
+        <f>Lines!$C$14&amp;IF(Inputs!$B$40,"",IF(Inputs!$B$36="",""," "&amp;Lines!$C$15))</f>
         <v/>
       </c>
       <c r="G5" s="10">
-        <f>IF(Inputs!$B$12="draw",Lines!$C$19,Lines!$C$18)</f>
+        <f>IF(Inputs!$B$12="draw",Lines!$C$18,Lines!$C$17)</f>
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>IF(Inputs!$B$6="","",Lines!$C$23)</f>
+        <f>IF(Inputs!$B$6="","",Lines!$C$22)</f>
         <v/>
       </c>
       <c r="I5" s="10">
@@ -1541,7 +1610,7 @@
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>status · making · edition + beneficiary · action</t>
+          <t>status · making · features + beneficiary · action</t>
         </is>
       </c>
       <c r="D6" s="10">
@@ -1549,15 +1618,15 @@
         <v/>
       </c>
       <c r="E6" s="10">
-        <f>Inputs!$B$24</f>
+        <f>Inputs!$B$29</f>
         <v/>
       </c>
       <c r="F6" s="10">
-        <f>IF(Inputs!$B$11&gt;1,Lines!$C$15,Lines!$C$14)&amp;IF(Inputs!$B$31="",""," "&amp;Lines!$C$16)</f>
+        <f>Lines!$C$14&amp;IF(Inputs!$B$36="",""," "&amp;Lines!$C$15)</f>
         <v/>
       </c>
       <c r="G6" s="10">
-        <f>IF(Inputs!$B$12="draw",Lines!$C$19,Lines!$C$18)</f>
+        <f>IF(Inputs!$B$12="draw",Lines!$C$18,Lines!$C$17)</f>
         <v/>
       </c>
       <c r="H6" s="10">
@@ -1584,23 +1653,23 @@
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>quote · status · edition + beneficiary · action</t>
+          <t>quote · status · features + beneficiary · action</t>
         </is>
       </c>
       <c r="D7" s="10">
-        <f>IF(Inputs!$B$25="","(no quote given, post skipped)",Lines!$C$8)</f>
+        <f>IF(Inputs!$B$30="","(no quote given, post skipped)",Lines!$C$8)</f>
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>IF(Inputs!$B$25="","",Lines!$C$9)</f>
+        <f>IF(Inputs!$B$30="","",Lines!$C$9)</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>IF(Inputs!$B$25="","",IF(Inputs!$B$11&gt;1,Lines!$C$15,Lines!$C$14)&amp;IF(Inputs!$B$31="",""," "&amp;Lines!$C$16))</f>
+        <f>IF(Inputs!$B$30="","",Lines!$C$14&amp;IF(Inputs!$B$36="",""," "&amp;Lines!$C$15))</f>
         <v/>
       </c>
       <c r="G7" s="10">
-        <f>IF(Inputs!$B$25="","",IF(Inputs!$B$12="draw",Lines!$C$19,Lines!$C$18))</f>
+        <f>IF(Inputs!$B$30="","",IF(Inputs!$B$12="draw",Lines!$C$18,Lines!$C$17))</f>
         <v/>
       </c>
       <c r="H7" s="10">
@@ -1608,7 +1677,7 @@
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>IF(Inputs!$B$25="","(no quote given, post skipped)",D7&amp;IF(E7="","",CHAR(10)&amp;CHAR(10)&amp;E7)&amp;IF(F7="","",CHAR(10)&amp;CHAR(10)&amp;F7)&amp;IF(G7="","",CHAR(10)&amp;CHAR(10)&amp;G7))</f>
+        <f>IF(Inputs!$B$30="","(no quote given, post skipped)",D7&amp;IF(E7="","",CHAR(10)&amp;CHAR(10)&amp;E7)&amp;IF(F7="","",CHAR(10)&amp;CHAR(10)&amp;F7)&amp;IF(G7="","",CHAR(10)&amp;CHAR(10)&amp;G7))</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -1627,7 +1696,7 @@
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>status · edition + beneficiary · action</t>
+          <t>status · features + beneficiary · action</t>
         </is>
       </c>
       <c r="D8" s="10">
@@ -1639,11 +1708,11 @@
         <v/>
       </c>
       <c r="F8" s="10">
-        <f>IF(Inputs!$B$12="draw","",IF(Inputs!$B$11&gt;1,Lines!$C$15,Lines!$C$14)&amp;IF(Inputs!$B$31="",""," "&amp;Lines!$C$16))</f>
+        <f>IF(Inputs!$B$12="draw","",Lines!$C$14&amp;IF(Inputs!$B$36="",""," "&amp;Lines!$C$15))</f>
         <v/>
       </c>
       <c r="G8" s="10">
-        <f>IF(Inputs!$B$12="draw","",IF(Inputs!$B$12="draw",Lines!$C$21,Lines!$C$20))</f>
+        <f>IF(Inputs!$B$12="draw","",IF(Inputs!$B$12="draw",Lines!$C$20,Lines!$C$19))</f>
         <v/>
       </c>
       <c r="H8" s="10">
@@ -1670,7 +1739,7 @@
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>status · edition + beneficiary · action</t>
+          <t>status · features + beneficiary · action</t>
         </is>
       </c>
       <c r="D9" s="10">
@@ -1682,11 +1751,11 @@
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>IF(Inputs!$B$12="draw","",IF(Inputs!$B$11&gt;1,Lines!$C$15,Lines!$C$14)&amp;IF(Inputs!$B$31="",""," "&amp;Lines!$C$16))</f>
+        <f>IF(Inputs!$B$12="draw","",Lines!$C$14&amp;IF(Inputs!$B$36="",""," "&amp;Lines!$C$15))</f>
         <v/>
       </c>
       <c r="G9" s="10">
-        <f>IF(Inputs!$B$12="draw","",IF(Inputs!$B$12="draw",Lines!$C$21,Lines!$C$20))</f>
+        <f>IF(Inputs!$B$12="draw","",IF(Inputs!$B$12="draw",Lines!$C$20,Lines!$C$19))</f>
         <v/>
       </c>
       <c r="H9" s="10">
@@ -1713,7 +1782,7 @@
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>status · edition + beneficiary · action</t>
+          <t>status · features + beneficiary · action</t>
         </is>
       </c>
       <c r="D10" s="10">
@@ -1725,11 +1794,11 @@
         <v/>
       </c>
       <c r="F10" s="10">
-        <f>IF(Inputs!$B$11&gt;1,Lines!$C$15,Lines!$C$14)&amp;IF(Inputs!$B$31="",""," "&amp;Lines!$C$16)</f>
+        <f>Lines!$C$14&amp;IF(Inputs!$B$36="",""," "&amp;Lines!$C$15)</f>
         <v/>
       </c>
       <c r="G10" s="10">
-        <f>IF(Inputs!$B$12="draw",Lines!$C$21,Lines!$C$20)</f>
+        <f>IF(Inputs!$B$12="draw",Lines!$C$20,Lines!$C$19)</f>
         <v/>
       </c>
       <c r="H10" s="10">
@@ -1778,7 +1847,7 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Every post is: status line, substance, edition line, action line, and a hashtag on the announcement only. Coming Soon opens with the bio because the bio names the artist.</t>
+          <t>Every post is: status line, substance, features line, action line, and a hashtag on the announcement only. Coming Soon opens with the bio because the bio names the artist.</t>
         </is>
       </c>
     </row>
@@ -1809,12 +1878,12 @@
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>Edition line</t>
+          <t>Features line</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Signed by the artist and individually numbered. The beneficiary is named once per post: in the edition line unless the hook already names it.</t>
+          <t>The release's features as short sentences: the standard three (signed by the artist, individually numbered, free worldwide shipping) plus anything bespoke. The beneficiary follows, named once per post.</t>
         </is>
       </c>
     </row>
@@ -1838,7 +1907,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Three per release, written once: bio (2 to 3 sentences), hook (1 to 2 sentences, shared with the email), making (one sentence naming Make-Ready). The quote is verbatim.</t>
+          <t>Three per release, written once: bio (2 to 3 sentences), hook (1 to 2 sentences about the work only, shared with the email), making (one sentence naming Make-Ready). The quote is verbatim. The hook and bio must not repeat each other; the templates place the beneficiary, the medium and the features.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Extend the email set to the advisor, artist and partner voices
Fragments are now voice-neutral, so the same hook and making line serve
the Insiders early-access email, the artist's own email, the partner's
email, the welcome email and edition-closed, alongside our own. A voice
filter adds "our" or "Avant Arte's" to the making line. One beneficiary
phrase everywhere, "released in support of". Spreadsheet synced.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KCpXfXvgVaMZkSdhMYLgwy
</commit_message>
<xml_diff>
--- a/tool/instagram-set.xlsx
+++ b/tool/instagram-set.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -889,16 +889,16 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>The Changeling portrays a child as a symbol of modern youth, exploring how technology shapes today's generations. Grayson describes the work as intentionally 'quite disturbing', a changeling reimagined for the digital age.</t>
+          <t>The Changeling portrays a child as a symbol of modern youth, exploring how technology shapes today's generations. It reimagines changeling folklore for the digital age, and is intended to be 'quite disturbing'.</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>1 to 2 sentences about the work only; the same hook the email uses. The templates place the beneficiary, the medium and the features.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="48" customHeight="1">
+          <t>1 to 2 sentences about the work only: no artist name, no we or our, so it also works in the artist's and partner's emails.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="32" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
           <t>making</t>
@@ -906,12 +906,12 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>To create the edition, our printmakers at Make-Ready (@make__ready) translated a new design into a 9-colour silkscreen, capturing the vivid detail of Grayson's drawing style.</t>
+          <t>To create the edition, printmakers at Make-Ready translated a new design into a 9-colour silkscreen, capturing the vivid detail of the original drawing.</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>one sentence on how it was made, naming Make-Ready. Sustain only.</t>
+          <t>one sentence on how it was made, written as 'printmakers at Make-Ready'; the sheet adds 'our' and the tag.</t>
         </is>
       </c>
     </row>
@@ -1054,14 +1054,30 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
+          <t>making_ours</t>
+        </is>
+      </c>
+      <c r="B40" s="9">
+        <f>SUBSTITUTE($B$29,"printmakers at Make-Ready","our printmakers at Make-Ready (@make__ready)")</f>
+        <v/>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>the making line in our voice, with the Make-Ready tag</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
           <t>hook_names_beneficiary</t>
         </is>
       </c>
-      <c r="B40" s="9">
+      <c r="B41" s="9">
         <f>IF($B$18="",FALSE,ISNUMBER(SEARCH($B$18,$B$28)))</f>
         <v/>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>TRUE when the hook already names the beneficiary, so the edition line will not</t>
         </is>
@@ -1579,7 +1595,7 @@
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>Lines!$C$14&amp;IF(Inputs!$B$40,"",IF(Inputs!$B$36="",""," "&amp;Lines!$C$15))</f>
+        <f>Lines!$C$14&amp;IF(Inputs!$B$41,"",IF(Inputs!$B$36="",""," "&amp;Lines!$C$15))</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -1618,7 +1634,7 @@
         <v/>
       </c>
       <c r="E6" s="10">
-        <f>Inputs!$B$29</f>
+        <f>Inputs!$B$40</f>
         <v/>
       </c>
       <c r="F6" s="10">
@@ -1907,7 +1923,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Three per release, written once: bio (2 to 3 sentences), hook (1 to 2 sentences about the work only, shared with the email), making (one sentence naming Make-Ready). The quote is verbatim. The hook and bio must not repeat each other; the templates place the beneficiary, the medium and the features.</t>
+          <t>Three per release, written once: bio (2 to 3 sentences), hook (1 to 2 sentences about the work only, shared with the email), making (one sentence naming Make-Ready). The quote is verbatim. The hook and bio must not repeat each other. Fragments are voice-neutral (no we or our, no artist name in the hook or making line) so the same lines serve the artist's and partner's emails.</t>
         </is>
       </c>
     </row>

</xml_diff>